<commit_message>
Add global packaging/manufacturing Oracle Fusion peer set
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLLBmgNKGat6rZHTm3o16N
</commit_message>
<xml_diff>
--- a/research/nordic-oracle-fusion-scan/nordic_oracle_fusion_scan_2026-10.xlsx
+++ b/research/nordic-oracle-fusion-scan/nordic_oracle_fusion_scan_2026-10.xlsx
@@ -8,18 +8,20 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="No signal found" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partners hiring" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search strings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global packaging peers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="No signal found" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partners hiring" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Search strings" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Accounts'!$A$1:$J$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Excluded'!$A$1:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'No signal found'!$A$1:$A$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Partners hiring'!$A$1:$C$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Search strings'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Global packaging peers'!$A$1:$I$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Accounts'!$A$1:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Excluded'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'No signal found'!$A$1:$A$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Partners hiring'!$A$1:$C$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Search strings'!$A$1:$B$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -590,6 +592,690 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>HQ</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Oracle status</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Fusion scope</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Prior system</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Theme match</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Tama Group</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Israel (10+ plants)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Agricultural packaging &amp; netting</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Fusion - implementing (TamaUP)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ERP, SCM &amp; Manufacturing, Procurement, HCM</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Oracle EBS</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>EBS-&gt;Fusion; multi-site consolidation</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>PwC case study, Jul 2026</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pwc.com/gx/en/services/alliances/oracle/tama-group-oracle-case-study.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Altium Packaging</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>US (Atlanta)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Rigid plastic packaging</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Fusion - implementing 2026</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Financials, EPM (finance-first)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Finance-first rollout</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Job ads: 2026 ERP Implementation - Oracle Fusion intern; IS Oracle Fusion Financials &amp; EPM Senior Manager; Sr Infrastructure Engineer Oracle Fusion</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>https://builtin.com/job/2026-erp-implementation-oracle-fusion-intern/7531387</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Litoplas</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Flexible plastic packaging</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Fusion - live</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>ERP + Maintenance</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Plant-floor use (maintenance)</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Oracle customer story (~2021)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/uk/customers/litoplas/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Unnamed German industrial packaging company</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Industrial packaging</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Fusion - live</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>ERP + EPM (PBCS)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Finance/EPM</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Oracle EPM use-case PDF (company not named)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>https://a.storyblok.com/f/291127619322886/x/c27f12542a/case-study-packaging.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Genpak</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>US (Charlotte)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Foodservice packaging (direct Huhtamaki competitor)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Oracle - product unconfirmed</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Verify EBS vs Fusion</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Supply Chain Analyst ad mentions Oracle upgrades / new modules</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ziprecruiter.com/Jobs/Fusion-Packaging</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Sonoco</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Consumer &amp; industrial packaging</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Oracle EBS (not Fusion)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>EBS on OCI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>EBS installed base - Fusion candidate</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Oracle architecture doc + HCLTech case</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>https://docs.oracle.com/en/solutions/sonoco-on-oci/index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Printpack</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Flexible packaging</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>JD Edwards; evaluated Oracle Cloud ERP</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>JDE</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Oracle base evaluating Fusion</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>erpresearch directory (third-party)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.erpresearch.com/erp-customers/oracle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Amcor (+Berry Global)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CH/US</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Flexible &amp; rigid packaging</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Not Oracle ERP (SAP; Berry on JDE)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SAP / JDE</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Orange Business case; directory</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.orange-business.com/en/case-study/amcor-consolidates-corporate-applications-orange-business-services-hybrid-cloud-greater</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>UCC Group</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Coffee manufacturing (process)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Fusion - live</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>ERP + SCM &amp; Manufacturing</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Global multi-entity</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Oracle customer story</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/customers/ucc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Cohu</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Semiconductor equipment</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Fusion - live</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>ERP, SCM, CX</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Acquisition integration</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Oracle SCM page story</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/scm/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Johnson Controls</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Building equipment</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Fusion - live</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Fusion Cloud (global ops)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Global multi-entity</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Oracle industrial manufacturing case list</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/europe/industrial-manufacturing/industrial-manufacturing-case-studies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Alcar Ruote</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Automotive wheels</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Fusion - live</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>ERP + SCM &amp; Manufacturing (planning, OM, procurement)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>legacy</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Full plant scope in Europe</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Oracle industrial manufacturing case</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/industrial-manufacturing/industrial-manufacturing-case-studies/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Vertiv</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Power &amp; cooling equipment</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Fusion - live</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>ERP + CPQ</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>EBS / IFS</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>EBS-&gt;Fusion; acquisitions</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Oracle customer story; job ad on IFS-&gt;Oracle migration</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oracle.com/customers/vertiv/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1559,7 +2245,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1743,7 +2429,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2006,7 +2692,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2281,7 +2967,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>